<commit_message>
v0.9.7: iki dilli arayüz ve İngilizce kod tabanı
Arayüz Türkçe/İngilizce çalışıyor; dil rol ekranından ve üst bardan
değiştiriliyor, seçim diske kaydediliyor. Sunucu mesajları da kataloğa
alındı, süren bir koşu dil değişince yeniden çevriliyor.

Kod tabanı, arayüz metinleri dışında tamamen İngilizce. IP koşusu
ilerlemesi serbest metin yerine yapılandırılmış olaylardan okunuyor;
Excel sütunları koda sabit kimliklerle bağlandı. Eski Türkçe ayar
dosyası göçü ve ölü kod kaldırıldı.
</commit_message>
<xml_diff>
--- a/Field_Device_Verification.xlsx
+++ b/Field_Device_Verification.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Kontrol Listesi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -663,7 +663,7 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Sarı hücreler elle doldurulur. Set numarası B1'e girilir; IP şablonlarındaki 'n' bu numaraya göre otomatik çözülür.</t>
+          <t>Yellow cells are filled in by hand. Enter the set number in B1; the 'n' in the IP templates resolves to it automatically.</t>
         </is>
       </c>
       <c r="D1" s="20" t="n"/>
@@ -690,7 +690,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>YATAKLI VAGON — SAHA CİHAZ DOĞRULAMA KONTROL LİSTESİ</t>
+          <t>SLEEPER COACH — FIELD DEVICE VERIFICATION CHECKLIST</t>
         </is>
       </c>
       <c r="B2" s="20" t="n"/>
@@ -719,14 +719,14 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>FİZİKSEL KONTROL</t>
+          <t>PHYSICAL CHECK</t>
         </is>
       </c>
       <c r="B3" s="20" t="n"/>
       <c r="C3" s="21" t="n"/>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>DOĞRULAMA KRİTERİ</t>
+          <t>VERIFICATION CRITERIA</t>
         </is>
       </c>
       <c r="E3" s="20" t="n"/>
@@ -735,7 +735,7 @@
       <c r="H3" s="21" t="n"/>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>YAZILIM KONTROL</t>
+          <t>SOFTWARE CHECK</t>
         </is>
       </c>
       <c r="J3" s="20" t="n"/>
@@ -756,7 +756,7 @@
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Bölüm</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -771,77 +771,77 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Cihaz Tanımı</t>
+          <t>Device definition</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>IP Şablonu</t>
+          <t>IP template</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Beklenen IP</t>
+          <t>Expected IP</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Beklenen Versiyon</t>
+          <t>Expected version</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Beklenen SIP Dahili No</t>
+          <t>Expected SIP extension</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Cihaz İsmi</t>
+          <t>Device name</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>Bağlantı Bilgisi</t>
+          <t>Connection info</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>Versiyon</t>
+          <t>Version</t>
         </is>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>Cihaz Numarası</t>
+          <t>Device number</t>
         </is>
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>Durum Açıklaması</t>
+          <t>Status description</t>
         </is>
       </c>
       <c r="N4" s="7" t="inlineStr">
         <is>
-          <t>Çalışma Süresi</t>
+          <t>Uptime</t>
         </is>
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>Hoparlör Ses Seviyesi</t>
+          <t>Speaker volume</t>
         </is>
       </c>
       <c r="P4" s="7" t="inlineStr">
         <is>
-          <t>Mikrofon Ses Seviyesi</t>
+          <t>Microphone volume</t>
         </is>
       </c>
       <c r="Q4" s="7" t="inlineStr">
         <is>
-          <t>Hoparlör Gain</t>
+          <t>Speaker gain</t>
         </is>
       </c>
       <c r="R4" s="7" t="inlineStr">
         <is>
-          <t>Mikrofon Gain</t>
+          <t>Microphone gain</t>
         </is>
       </c>
       <c r="S4" s="7" t="inlineStr">
@@ -851,29 +851,29 @@
       </c>
       <c r="T4" s="7" t="inlineStr">
         <is>
-          <t>SIP Dahili No</t>
+          <t>SIP extension</t>
         </is>
       </c>
       <c r="U4" s="7" t="inlineStr">
         <is>
-          <t>SIP Arama No</t>
+          <t>SIP outbound number</t>
         </is>
       </c>
       <c r="V4" s="7" t="inlineStr">
         <is>
-          <t>Saat Dilimi</t>
+          <t>Time zone</t>
         </is>
       </c>
       <c r="W4" s="7" t="inlineStr">
         <is>
-          <t>Ağ/Zaman Kontrolü</t>
+          <t>Network/time check</t>
         </is>
       </c>
     </row>
     <row r="5" ht="19" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SWITCH   ·   2 kayıt</t>
+          <t xml:space="preserve">  SWITCH   ·   2 records</t>
         </is>
       </c>
       <c r="B5" s="20" t="n"/>
@@ -990,7 +990,7 @@
     <row r="8" ht="19" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PISCU   ·   1 kayıt</t>
+          <t xml:space="preserve">  PISCU   ·   1 records</t>
         </is>
       </c>
       <c r="B8" s="20" t="n"/>
@@ -1065,7 +1065,7 @@
     <row r="10" ht="19" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ICU   ·   1 kayıt</t>
+          <t xml:space="preserve">  ICU   ·   1 records</t>
         </is>
       </c>
       <c r="B10" s="20" t="n"/>
@@ -1140,7 +1140,7 @@
     <row r="12" ht="19" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  HMI   ·   1 kayıt</t>
+          <t xml:space="preserve">  HMI   ·   1 records</t>
         </is>
       </c>
       <c r="B12" s="20" t="n"/>
@@ -1215,7 +1215,7 @@
     <row r="14" ht="19" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AP (Access Point)   ·   2 kayıt</t>
+          <t xml:space="preserve">  AP (Access Point)   ·   2 records</t>
         </is>
       </c>
       <c r="B14" s="20" t="n"/>
@@ -1336,7 +1336,7 @@
     <row r="17" ht="19" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  LED · Front   ·   2 kayıt</t>
+          <t xml:space="preserve">  LED · Front   ·   2 records</t>
         </is>
       </c>
       <c r="B17" s="20" t="n"/>
@@ -1457,7 +1457,7 @@
     <row r="20" ht="19" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  LCD · Landing   ·   2 kayıt</t>
+          <t xml:space="preserve">  LCD · Landing   ·   2 records</t>
         </is>
       </c>
       <c r="B20" s="20" t="n"/>
@@ -1578,7 +1578,7 @@
     <row r="23" ht="19" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  LCD · Compartment   ·   11 kayıt   ·   ek alan: Saat Dilimi, SIP PBX IP, SIP Dahili No</t>
+          <t xml:space="preserve">  LCD · Compartment   ·   11 records   ·   extra field: Time zone, SIP PBX IP, SIP extension</t>
         </is>
       </c>
       <c r="B23" s="20" t="n"/>
@@ -2157,7 +2157,7 @@
     <row r="35" ht="19" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Announcement · UIC   ·   1 kayıt   ·   ek alan: SIP PBX IP, SIP Dahili No</t>
+          <t xml:space="preserve">  Announcement · UIC   ·   1 records   ·   extra field: SIP PBX IP, SIP extension</t>
         </is>
       </c>
       <c r="B35" s="20" t="n"/>
@@ -2236,7 +2236,7 @@
     <row r="37" ht="19" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Announcement · Amplifier   ·   1 kayıt   ·   ek alan: Hoparlör Ses Seviyesi, Mikrofon Ses Seviyesi, Hoparlör Gain, Mikrofon Gain, SIP PBX IP, SIP Dahili No</t>
+          <t xml:space="preserve">  Announcement · Amplifier   ·   1 records   ·   extra field: Speaker volume, Microphone volume, Speaker gain, Microphone gain, SIP PBX IP, SIP extension</t>
         </is>
       </c>
       <c r="B37" s="20" t="n"/>
@@ -2315,7 +2315,7 @@
     <row r="39" ht="19" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Announcement · Handset   ·   1 kayıt   ·   ek alan: Hoparlör Ses Seviyesi, Mikrofon Ses Seviyesi, Hoparlör Gain, Mikrofon Gain, SIP PBX IP, SIP Dahili No, SIP Arama No</t>
+          <t xml:space="preserve">  Announcement · Handset   ·   1 records   ·   extra field: Speaker volume, Microphone volume, Speaker gain, Microphone gain, SIP PBX IP, SIP extension, SIP outbound number</t>
         </is>
       </c>
       <c r="B39" s="20" t="n"/>
@@ -2394,7 +2394,7 @@
     <row r="41" ht="19" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Announcement · Intercom   ·   12 kayıt   ·   ek alan: Hoparlör Ses Seviyesi, Mikrofon Ses Seviyesi, Hoparlör Gain, Mikrofon Gain, SIP PBX IP, SIP Dahili No, SIP Arama No</t>
+          <t xml:space="preserve">  Announcement · Intercom   ·   12 records   ·   extra field: Speaker volume, Microphone volume, Speaker gain, Microphone gain, SIP PBX IP, SIP extension, SIP outbound number</t>
         </is>
       </c>
       <c r="B41" s="20" t="n"/>
@@ -3023,7 +3023,7 @@
     <row r="54" ht="19" customHeight="1">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Camera · Corridor   ·   2 kayıt   ·   ek alan: Ağ/Zaman Kontrolü</t>
+          <t xml:space="preserve">  Camera · Corridor   ·   2 records   ·   extra field: Network/time check</t>
         </is>
       </c>
       <c r="B54" s="20" t="n"/>
@@ -3144,7 +3144,7 @@
     <row r="57" ht="19" customHeight="1">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Camera · Landing   ·   2 kayıt   ·   ek alan: Ağ/Zaman Kontrolü</t>
+          <t xml:space="preserve">  Camera · Landing   ·   2 records   ·   extra field: Network/time check</t>
         </is>
       </c>
       <c r="B57" s="20" t="n"/>
@@ -3265,7 +3265,7 @@
     <row r="60" ht="19" customHeight="1">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NVR   ·   1 kayıt   ·   ek alan: Ağ/Zaman Kontrolü</t>
+          <t xml:space="preserve">  NVR   ·   1 records   ·   extra field: Network/time check</t>
         </is>
       </c>
       <c r="B60" s="20" t="n"/>
@@ -3337,10 +3337,12 @@
       <c r="V61" s="14" t="n"/>
       <c r="W61" s="15" t="n"/>
     </row>
+    <row r="62"/>
+    <row r="63"/>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>SONUÇ</t>
+          <t>RESULT</t>
         </is>
       </c>
       <c r="B64" s="20" t="n"/>
@@ -3369,7 +3371,7 @@
     <row r="65" ht="16" customHeight="1">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>Toplam Kayıt</t>
+          <t>Total records</t>
         </is>
       </c>
       <c r="B65" s="19">
@@ -3378,7 +3380,7 @@
       </c>
       <c r="C65" s="18" t="inlineStr">
         <is>
-          <t>Versiyon Girilmeyen</t>
+          <t>Version missing</t>
         </is>
       </c>
       <c r="D65" s="19">
@@ -3387,7 +3389,7 @@
       </c>
       <c r="E65" s="18" t="inlineStr">
         <is>
-          <t>Bağlantı Bekleyen</t>
+          <t>Awaiting connection</t>
         </is>
       </c>
       <c r="F65" s="19">
@@ -3396,29 +3398,29 @@
       </c>
       <c r="G65" s="18" t="inlineStr">
         <is>
-          <t>Aktif</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H65" s="19">
-        <f>COUNTIF(M6:M61,"Aktif")</f>
+        <f>COUNTIF(M6:M61,"Active")</f>
         <v/>
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>Pasif</t>
+          <t>Inactive</t>
         </is>
       </c>
       <c r="J65" s="19">
-        <f>COUNTIF(M6:M61,"Pasif*")</f>
+        <f>COUNTIF(M6:M61,"Inactive*")</f>
         <v/>
       </c>
       <c r="K65" s="18" t="inlineStr">
         <is>
-          <t>Genel Sonuç</t>
+          <t>Overall result</t>
         </is>
       </c>
       <c r="L65" s="19">
-        <f>IF(COUNTIF(M6:M61,"Pasif*")&gt;0,"UYGUN DEĞİL",IF(COUNTA(J6:J61)&lt;COUNTIF(A6:A61,"Yataklı"),"KONTROL BEKLİYOR","UYGUN"))</f>
+        <f>IF(COUNTIF(M6:M61,"Inactive*")&gt;0,"NOT COMPLIANT",IF(COUNTA(J6:J61)&lt;COUNTIF(A6:A61,"Yataklı"),"AWAITING CHECK","COMPLIANT"))</f>
         <v/>
       </c>
       <c r="M65" s="20" t="n"/>

</xml_diff>